<commit_message>
Add 5 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (22):
- blocks/cards-teaser/cards-teaser.css
- blocks/columns-info/columns-info.css
- blocks/header/header.css
- blocks/header/header.js
- blocks/hero-corporate/hero-corporate.css
- blocks/hero-corporate/hero-corporate.js
- blocks/hero-corporate/metadata.json
- blocks/tabs-product/tabs-product.css
- fonts/aig-icons.ttf
- fonts/aig-icons.woff
- package-lock.json
- package.json
- styles/styles.css
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/parsers/hero-corporate.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/sonpo.report.json
- tools/importer/run-import-bypass-csp.cjs
- tools/importer/run-import-bypass-csp.js
- tools/importer/transformers/aig-cleanup.js
- tools/importer/urls-homepage.txt
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>errorStack</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -43,6 +49,9 @@
     <t>["hero-corporate","columns-info","columns-info","columns-info","columns-info","columns-info","columns-info","columns-info","columns-info","columns-info","columns-info","columns-info","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","tabs-product"]</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>index</t>
   </si>
   <si>
@@ -59,6 +68,31 @@
   </si>
   <si>
     <t>https://www.aig.co.jp/</t>
+  </si>
+  <si>
+    <t>sonpo.report.json</t>
+  </si>
+  <si>
+    <t>CustomImportScript.default not found after 10s. The bundled script may not have loaded correctly. Check browser console for errors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error: CustomImportScript.default not found after 10s. The bundled script may not have loaded correctly. Check browser console for errors.
+    at processUrl (file:///home/node/.claude/plugins/cache/excat-marketplace/excat/2.1.1/skills/excat-content-import/scripts/run-bulk-import.js:293:13)
+    at runNextTicks (node:internal/process/task_queues:65:5)
+    at process.processImmediate (node:internal/timers:472:9)
+    at async main (file:///home/node/.claude/plugins/cache/excat-marketplace/excat/2.1.1/skills/excat-content-import/scripts/run-bulk-import.js:457:22)</t>
+  </si>
+  <si>
+    <t>sonpo</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-03-05T15:57:08.462Z</t>
+  </si>
+  <si>
+    <t>https://www.aig.co.jp/sonpo</t>
   </si>
 </sst>
 </file>
@@ -447,19 +481,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="27" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="2" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="27" customWidth="1"/>
+    <col min="10" max="10" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,35 +518,79 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>